<commit_message>
Date flip detection, GSTIN guard, vendor onboarding scripts
</commit_message>
<xml_diff>
--- a/Vendor-Ledgers.xlsx
+++ b/Vendor-Ledgers.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="41" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2869,6 +2869,215 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Campus Mall</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Staff Welfare</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>d943a326-ab2e-49fc-b81d-38b1c1cffcf9</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>5589375000001971210</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>23AAECC8161B1Z4</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>5589375000000502039</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>DAFFODIL</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Boarding &amp; Lodging Expenses</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>757e2cda-e97d-4b69-bd0d-26a4ca40eee6</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>5589375000001092133</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>29AQSPK3233B1ZV</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>5589375000000120713</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>THEEMINENCE TECHNOLOGY SOLUTIONS</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Software Development &amp; Technical consultancy</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>52277a54-612b-4552-99d7-d62a1a937542</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>5589375000002852145</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>33AALFT3018J1Z6</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>5589375000003097040</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Md Faizan Ansari</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Software Development &amp; Technical consultancy</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>37f75ec0-a0b9-4301-bbcc-1172c1420dfb</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>5589375000003225058</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>5589375000003097040</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>True Value Textile</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Staff Welfare</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>fa606a2f-6aba-4288-87ce-ea822dc72ce1</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>5589375000003612205</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>33DALPK5489M2ZX</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>5589375000000502039</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Jake Canning</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Consultancy Fee - I/S @ 2% TDS</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>68a9da82-be46-4577-b55e-299450574b45</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>5589375000001879001</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>5589375000000120635</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>V SATYA SUJATA</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Professional Charges - Un Registered</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>79ed84ae-8cbc-44b1-81d2-86b882bcafe0</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>5589375000002339001</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>5589375000000120677</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update database with manual approved invoices
</commit_message>
<xml_diff>
--- a/Vendor-Ledgers.xlsx
+++ b/Vendor-Ledgers.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="41" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3078,6 +3078,33 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Rabbani Kaja Mohideen</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Software Development &amp; Technical Manpower Charges</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>6c57a49b-ac8a-4828-8cbc-92c38c2794f1</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>5589375000004070436</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>5589375000003097044</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>